<commit_message>
feat: Iniciado o processo de cadastro dos clientes
</commit_message>
<xml_diff>
--- a/ERP_Portal_Fake/Sistema_Integrador_Portal_Fake/Planilha_Mestra.xlsx
+++ b/ERP_Portal_Fake/Sistema_Integrador_Portal_Fake/Planilha_Mestra.xlsx
@@ -523,15 +523,15 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>CONCLUIDO_P2</t>
+          <t>DUPLICADO_P3</t>
         </is>
       </c>
       <c r="H2" s="3" t="n">
-        <v>46251.69543553241</v>
+        <v>46251.71147211806</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Documentação validada e integrada via RPA</t>
+          <t>Documentação validada e integrada via RPA | CPF já cadastrado previamente no Portal Fake | CPF já cadastrado previamente no Portal Fake</t>
         </is>
       </c>
     </row>
@@ -552,7 +552,6 @@
           <t>Rua H, 149 - Bairro Flores - Manaus/AM</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
           <t>(92) 99008-1008</t>
@@ -560,21 +559,63 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>CONCLUIDO_P2</t>
+          <t>DUPLICADO_P3</t>
         </is>
       </c>
       <c r="H3" s="3" t="n">
-        <v>46251.69543876505</v>
+        <v>46251.71147710648</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Protocolo: #PROT-20260729-0003</t>
+          <t>Protocolo: #PROT-20260729-0003 | Falha no portal: Exceção durante cadastro no portal: Page.wait_for_selector: Timeout 4000ms exceeded.
+Call log:
+  - waiting for locator("#modal[hidden]") to be visible
+    12 × locator resolved to hidden &lt;div hidden="" id="modal" class="modal" aria-hidden="true"&gt;…&lt;/div&gt; | CPF já cadastrado previamente no Portal Fake</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="C4" s="2" t="n"/>
-      <c r="H4" s="3" t="n"/>
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>22233344455</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Mariana Souza</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>33739</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Av. Djalma Batista, 500 - Flores - Manaus/AM</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>mariana.souza@empresa.com</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>(92) 98123-4567</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>CONCLUIDO_P3</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>46251.71167067454</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Processado via RPA P2 | Cadastrado com sucesso no Portal Fake via RPA</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="C5" s="2" t="n"/>

</xml_diff>